<commit_message>
feat: 100 yeni kelime (301-400) — set 400/400
Gercek Turkce kelime kanca, kanca ile anlam birbirine bir sey yapiyor
(dog ≈ dag: "Kopek daga tirmandi", boss ≈ bos, kind ≈ kaynana...).
tools/yeni-kelimeler.mjs aday tablosunu uretir ve bir kartin kancasinin
baska kartin anlami olmasini (honey ≈ hani / ball ≈ bal) setle birlikte
denetler. 100 gorsel + 9 yeniden = 8.175 kredi; recetede dort yeni ders.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kart-havuzu-300.xlsx
+++ b/kart-havuzu-300.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2123" uniqueCount="1396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2923" uniqueCount="1788">
   <si>
     <t>#</t>
   </si>
@@ -4181,7 +4181,1183 @@
     <t>Tekerlekli paten</t>
   </si>
   <si>
-    <t>KART HAVUZU — 300 KART</t>
+    <t>dog</t>
+  </si>
+  <si>
+    <t>köpek</t>
+  </si>
+  <si>
+    <t>dağ</t>
+  </si>
+  <si>
+    <t>Köpek dağa tırmandı</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>money</t>
+  </si>
+  <si>
+    <t>para</t>
+  </si>
+  <si>
+    <t>mani</t>
+  </si>
+  <si>
+    <t>Mani okuyana para attılar</t>
+  </si>
+  <si>
+    <t>friend</t>
+  </si>
+  <si>
+    <t>arkadaş</t>
+  </si>
+  <si>
+    <t>frenk</t>
+  </si>
+  <si>
+    <t>Arkadaşım frenk üzümü getirdi</t>
+  </si>
+  <si>
+    <t>face</t>
+  </si>
+  <si>
+    <t>yüz</t>
+  </si>
+  <si>
+    <t>fes</t>
+  </si>
+  <si>
+    <t>Yüzüne fes düştü</t>
+  </si>
+  <si>
+    <t>hand</t>
+  </si>
+  <si>
+    <t>el</t>
+  </si>
+  <si>
+    <t>hendek</t>
+  </si>
+  <si>
+    <t>Hendekten bir el uzandı</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>ad</t>
+  </si>
+  <si>
+    <t>nem</t>
+  </si>
+  <si>
+    <t>Adını nemli cama yazdı</t>
+  </si>
+  <si>
+    <t>book</t>
+  </si>
+  <si>
+    <t>kitap</t>
+  </si>
+  <si>
+    <t>bük</t>
+  </si>
+  <si>
+    <t>Kitabı ikiye büktü</t>
+  </si>
+  <si>
+    <t>bed</t>
+  </si>
+  <si>
+    <t>yatak</t>
+  </si>
+  <si>
+    <t>bedava</t>
+  </si>
+  <si>
+    <t>Bedava yatağa herkes atladı</t>
+  </si>
+  <si>
+    <t>chair</t>
+  </si>
+  <si>
+    <t>sandalye</t>
+  </si>
+  <si>
+    <t>çay</t>
+  </si>
+  <si>
+    <t>Sandalyeye çay döküldü</t>
+  </si>
+  <si>
+    <t>wall</t>
+  </si>
+  <si>
+    <t>duvar</t>
+  </si>
+  <si>
+    <t>voleybol</t>
+  </si>
+  <si>
+    <t>Duvara karşı voleybol oynadı</t>
+  </si>
+  <si>
+    <t>girl</t>
+  </si>
+  <si>
+    <t>kız</t>
+  </si>
+  <si>
+    <t>gül</t>
+  </si>
+  <si>
+    <t>Kız gülü kokladı</t>
+  </si>
+  <si>
+    <t>bus</t>
+  </si>
+  <si>
+    <t>otobüs</t>
+  </si>
+  <si>
+    <t>bas</t>
+  </si>
+  <si>
+    <t>Gaza bas, otobüse yetiş!</t>
+  </si>
+  <si>
+    <t>town</t>
+  </si>
+  <si>
+    <t>kasaba</t>
+  </si>
+  <si>
+    <t>tavan</t>
+  </si>
+  <si>
+    <t>Tavanda bir kasaba var</t>
+  </si>
+  <si>
+    <t>rain</t>
+  </si>
+  <si>
+    <t>yağmur</t>
+  </si>
+  <si>
+    <t>ren geyiği</t>
+  </si>
+  <si>
+    <t>Ren geyiği yağmurda ıslandı</t>
+  </si>
+  <si>
+    <t>fire</t>
+  </si>
+  <si>
+    <t>ateş</t>
+  </si>
+  <si>
+    <t>fayans</t>
+  </si>
+  <si>
+    <t>Ateş fayansı çatlattı</t>
+  </si>
+  <si>
+    <t>ice</t>
+  </si>
+  <si>
+    <t>buz</t>
+  </si>
+  <si>
+    <t>ayaz</t>
+  </si>
+  <si>
+    <t>Ayazda su buz tuttu</t>
+  </si>
+  <si>
+    <t>shop</t>
+  </si>
+  <si>
+    <t>dükkân</t>
+  </si>
+  <si>
+    <t>şapşal</t>
+  </si>
+  <si>
+    <t>Şapşal satıcı dükkânı dağıttı</t>
+  </si>
+  <si>
+    <t>job</t>
+  </si>
+  <si>
+    <t>iş</t>
+  </si>
+  <si>
+    <t>cop</t>
+  </si>
+  <si>
+    <t>İş görüşmesine copla geldi</t>
+  </si>
+  <si>
+    <t>boss</t>
+  </si>
+  <si>
+    <t>patron</t>
+  </si>
+  <si>
+    <t>boş</t>
+  </si>
+  <si>
+    <t>Patronun koltuğu boş</t>
+  </si>
+  <si>
+    <t>pay</t>
+  </si>
+  <si>
+    <t>ödemek</t>
+  </si>
+  <si>
+    <t>Payını öde</t>
+  </si>
+  <si>
+    <t>take</t>
+  </si>
+  <si>
+    <t>almak</t>
+  </si>
+  <si>
+    <t>tek</t>
+  </si>
+  <si>
+    <t>Pastadan tek dilim al</t>
+  </si>
+  <si>
+    <t>send</t>
+  </si>
+  <si>
+    <t>göndermek</t>
+  </si>
+  <si>
+    <t>senet</t>
+  </si>
+  <si>
+    <t>Senedi postayla gönderdi</t>
+  </si>
+  <si>
+    <t>help</t>
+  </si>
+  <si>
+    <t>yardım etmek</t>
+  </si>
+  <si>
+    <t>helva</t>
+  </si>
+  <si>
+    <t>Helva karıştırana yardım et</t>
+  </si>
+  <si>
+    <t>find</t>
+  </si>
+  <si>
+    <t>bulmak</t>
+  </si>
+  <si>
+    <t>fındık</t>
+  </si>
+  <si>
+    <t>Kayıp fındığı buldum</t>
+  </si>
+  <si>
+    <t>clean</t>
+  </si>
+  <si>
+    <t>temizlemek</t>
+  </si>
+  <si>
+    <t>kilim</t>
+  </si>
+  <si>
+    <t>Kilimi fırçayla temizledi</t>
+  </si>
+  <si>
+    <t>sleep</t>
+  </si>
+  <si>
+    <t>uyumak</t>
+  </si>
+  <si>
+    <t>slip</t>
+  </si>
+  <si>
+    <t>Slipiyle uyuyakaldı</t>
+  </si>
+  <si>
+    <t>catch</t>
+  </si>
+  <si>
+    <t>yakalamak</t>
+  </si>
+  <si>
+    <t>kaç</t>
+  </si>
+  <si>
+    <t>Kaç kaç, yakalayacak!</t>
+  </si>
+  <si>
+    <t>fall</t>
+  </si>
+  <si>
+    <t>düşmek</t>
+  </si>
+  <si>
+    <t>fal</t>
+  </si>
+  <si>
+    <t>Fal bakarken sandalyeden düştü</t>
+  </si>
+  <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>saymak</t>
+  </si>
+  <si>
+    <t>kont</t>
+  </si>
+  <si>
+    <t>Kont altınlarını saydı</t>
+  </si>
+  <si>
+    <t>wish</t>
+  </si>
+  <si>
+    <t>dilek</t>
+  </si>
+  <si>
+    <t>vişne</t>
+  </si>
+  <si>
+    <t>Vişne yerken dilek tuttu</t>
+  </si>
+  <si>
+    <t>hungry</t>
+  </si>
+  <si>
+    <t>aç</t>
+  </si>
+  <si>
+    <t>hangar</t>
+  </si>
+  <si>
+    <t>Aç pilot hangarda yemek arıyor</t>
+  </si>
+  <si>
+    <t>busy</t>
+  </si>
+  <si>
+    <t>meşgul</t>
+  </si>
+  <si>
+    <t>bizi</t>
+  </si>
+  <si>
+    <t>Bizi rahatsız etme, meşgulüz</t>
+  </si>
+  <si>
+    <t>young</t>
+  </si>
+  <si>
+    <t>genç</t>
+  </si>
+  <si>
+    <t>yangın</t>
+  </si>
+  <si>
+    <t>Genç itfaiyeci yangını söndürdü</t>
+  </si>
+  <si>
+    <t>kind</t>
+  </si>
+  <si>
+    <t>nazik</t>
+  </si>
+  <si>
+    <t>kaynana</t>
+  </si>
+  <si>
+    <t>Kaynana çok nazik çıktı</t>
+  </si>
+  <si>
+    <t>lazy</t>
+  </si>
+  <si>
+    <t>tembel</t>
+  </si>
+  <si>
+    <t>leziz</t>
+  </si>
+  <si>
+    <t>Tembel kedi leziz balığa bile kalkmadı</t>
+  </si>
+  <si>
+    <t>wet</t>
+  </si>
+  <si>
+    <t>ıslak</t>
+  </si>
+  <si>
+    <t>veteriner</t>
+  </si>
+  <si>
+    <t>Veteriner ıslak köpeği kuruladı</t>
+  </si>
+  <si>
+    <t>loud</t>
+  </si>
+  <si>
+    <t>yüksek sesli</t>
+  </si>
+  <si>
+    <t>lavta</t>
+  </si>
+  <si>
+    <t>Lavta çok yüksek sesli çaldı</t>
+  </si>
+  <si>
+    <t>sour</t>
+  </si>
+  <si>
+    <t>ekşi</t>
+  </si>
+  <si>
+    <t>savur</t>
+  </si>
+  <si>
+    <t>Ekşi limonu savurdu</t>
+  </si>
+  <si>
+    <t>fast</t>
+  </si>
+  <si>
+    <t>hızlı</t>
+  </si>
+  <si>
+    <t>fasıl</t>
+  </si>
+  <si>
+    <t>Fasılda saz hızlandı</t>
+  </si>
+  <si>
+    <t>apple</t>
+  </si>
+  <si>
+    <t>elma</t>
+  </si>
+  <si>
+    <t>apal</t>
+  </si>
+  <si>
+    <t>Apal apal elmaya bakıyor</t>
+  </si>
+  <si>
+    <t>egg</t>
+  </si>
+  <si>
+    <t>yumurta</t>
+  </si>
+  <si>
+    <t>eğe</t>
+  </si>
+  <si>
+    <t>Yumurtayı eğeyle törpüledi</t>
+  </si>
+  <si>
+    <t>rice</t>
+  </si>
+  <si>
+    <t>pirinç</t>
+  </si>
+  <si>
+    <t>ray</t>
+  </si>
+  <si>
+    <t>Pirinç raylara döküldü</t>
+  </si>
+  <si>
+    <t>soup</t>
+  </si>
+  <si>
+    <t>çorba</t>
+  </si>
+  <si>
+    <t>süpürge</t>
+  </si>
+  <si>
+    <t>Çorbayı süpürgeyle karıştırdı</t>
+  </si>
+  <si>
+    <t>oil</t>
+  </si>
+  <si>
+    <t>yağ</t>
+  </si>
+  <si>
+    <t>oy</t>
+  </si>
+  <si>
+    <t>Yağ şişesini oy sandığına attı</t>
+  </si>
+  <si>
+    <t>knife</t>
+  </si>
+  <si>
+    <t>bıçak</t>
+  </si>
+  <si>
+    <t>ney</t>
+  </si>
+  <si>
+    <t>Bıçakla ney yonttu</t>
+  </si>
+  <si>
+    <t>cow</t>
+  </si>
+  <si>
+    <t>inek</t>
+  </si>
+  <si>
+    <t>kavun</t>
+  </si>
+  <si>
+    <t>İnek kavunu yedi</t>
+  </si>
+  <si>
+    <t>horse</t>
+  </si>
+  <si>
+    <t>at</t>
+  </si>
+  <si>
+    <t>horoz</t>
+  </si>
+  <si>
+    <t>Horoz atın sırtına bindi</t>
+  </si>
+  <si>
+    <t>sheep</t>
+  </si>
+  <si>
+    <t>koyun</t>
+  </si>
+  <si>
+    <t>şipşak</t>
+  </si>
+  <si>
+    <t>Koyunun şipşak fotoğrafını çektim</t>
+  </si>
+  <si>
+    <t>ant</t>
+  </si>
+  <si>
+    <t>karınca</t>
+  </si>
+  <si>
+    <t>Karıncalar ant içti</t>
+  </si>
+  <si>
+    <t>owl</t>
+  </si>
+  <si>
+    <t>baykuş</t>
+  </si>
+  <si>
+    <t>avlu</t>
+  </si>
+  <si>
+    <t>Baykuş avluya kondu</t>
+  </si>
+  <si>
+    <t>tooth</t>
+  </si>
+  <si>
+    <t>tuş</t>
+  </si>
+  <si>
+    <t>Dişiyle tuşa bastı</t>
+  </si>
+  <si>
+    <t>cheek</t>
+  </si>
+  <si>
+    <t>yanak</t>
+  </si>
+  <si>
+    <t>çikolata</t>
+  </si>
+  <si>
+    <t>Yanağına çikolata bulaştı</t>
+  </si>
+  <si>
+    <t>body</t>
+  </si>
+  <si>
+    <t>vücut</t>
+  </si>
+  <si>
+    <t>bodur</t>
+  </si>
+  <si>
+    <t>Bodur adam vücut geliştirdi</t>
+  </si>
+  <si>
+    <t>roof</t>
+  </si>
+  <si>
+    <t>çatı</t>
+  </si>
+  <si>
+    <t>ruh</t>
+  </si>
+  <si>
+    <t>Çatıda bir ruh dolaşıyor</t>
+  </si>
+  <si>
+    <t>lake</t>
+  </si>
+  <si>
+    <t>göl</t>
+  </si>
+  <si>
+    <t>leke</t>
+  </si>
+  <si>
+    <t>Göle leke düştü</t>
+  </si>
+  <si>
+    <t>hat</t>
+  </si>
+  <si>
+    <t>hattat</t>
+  </si>
+  <si>
+    <t>Hattat şapkasına yazı yazdı</t>
+  </si>
+  <si>
+    <t>ring</t>
+  </si>
+  <si>
+    <t>yüzük</t>
+  </si>
+  <si>
+    <t>Boksör ringde yüzüğünü kaybetti</t>
+  </si>
+  <si>
+    <t>boot</t>
+  </si>
+  <si>
+    <t>çizme</t>
+  </si>
+  <si>
+    <t>but</t>
+  </si>
+  <si>
+    <t>Çizmeyi butuna kadar çekti</t>
+  </si>
+  <si>
+    <t>toy</t>
+  </si>
+  <si>
+    <t>oyuncak</t>
+  </si>
+  <si>
+    <t>Toy çocuk oyuncağını kırdı</t>
+  </si>
+  <si>
+    <t>doll</t>
+  </si>
+  <si>
+    <t>oyuncak bebek</t>
+  </si>
+  <si>
+    <t>dolma</t>
+  </si>
+  <si>
+    <t>Oyuncak bebek dolma yiyor</t>
+  </si>
+  <si>
+    <t>mirror</t>
+  </si>
+  <si>
+    <t>ayna</t>
+  </si>
+  <si>
+    <t>miras</t>
+  </si>
+  <si>
+    <t>Dedemden ayna miras kaldı</t>
+  </si>
+  <si>
+    <t>soap</t>
+  </si>
+  <si>
+    <t>sabun</t>
+  </si>
+  <si>
+    <t>sopa</t>
+  </si>
+  <si>
+    <t>Sabunu sopayla vurdu</t>
+  </si>
+  <si>
+    <t>bird</t>
+  </si>
+  <si>
+    <t>kuş</t>
+  </si>
+  <si>
+    <t>börek</t>
+  </si>
+  <si>
+    <t>Kuş böreği kapıp kaçtı</t>
+  </si>
+  <si>
+    <t>smile</t>
+  </si>
+  <si>
+    <t>gülümsemek</t>
+  </si>
+  <si>
+    <t>İsmail</t>
+  </si>
+  <si>
+    <t>İsmail hep gülümsüyor</t>
+  </si>
+  <si>
+    <t>tent</t>
+  </si>
+  <si>
+    <t>çadır</t>
+  </si>
+  <si>
+    <t>tente</t>
+  </si>
+  <si>
+    <t>Çadırın üstüne tente gerdi</t>
+  </si>
+  <si>
+    <t>tower</t>
+  </si>
+  <si>
+    <t>kule</t>
+  </si>
+  <si>
+    <t>tava</t>
+  </si>
+  <si>
+    <t>Kulenin tepesine tava koydular</t>
+  </si>
+  <si>
+    <t>lock</t>
+  </si>
+  <si>
+    <t>kilit</t>
+  </si>
+  <si>
+    <t>lokma</t>
+  </si>
+  <si>
+    <t>Kilide lokma sıkıştı</t>
+  </si>
+  <si>
+    <t>hammer</t>
+  </si>
+  <si>
+    <t>çekiç</t>
+  </si>
+  <si>
+    <t>hamur</t>
+  </si>
+  <si>
+    <t>Çekiçle hamuru dövdü</t>
+  </si>
+  <si>
+    <t>cage</t>
+  </si>
+  <si>
+    <t>kafes</t>
+  </si>
+  <si>
+    <t>keçe</t>
+  </si>
+  <si>
+    <t>Kafesi keçeyle örttü</t>
+  </si>
+  <si>
+    <t>tail</t>
+  </si>
+  <si>
+    <t>kuyruk</t>
+  </si>
+  <si>
+    <t>teyel</t>
+  </si>
+  <si>
+    <t>Kuyruğuna teyel attı</t>
+  </si>
+  <si>
+    <t>hide</t>
+  </si>
+  <si>
+    <t>saklanmak</t>
+  </si>
+  <si>
+    <t>hayda</t>
+  </si>
+  <si>
+    <t>Hayda, kedi yine saklandı!</t>
+  </si>
+  <si>
+    <t>tie</t>
+  </si>
+  <si>
+    <t>bağlamak</t>
+  </si>
+  <si>
+    <t>tay</t>
+  </si>
+  <si>
+    <t>Tayı ağaca bağladı</t>
+  </si>
+  <si>
+    <t>dig</t>
+  </si>
+  <si>
+    <t>kazmak</t>
+  </si>
+  <si>
+    <t>dik</t>
+  </si>
+  <si>
+    <t>Dik bir çukur kazdı</t>
+  </si>
+  <si>
+    <t>melt</t>
+  </si>
+  <si>
+    <t>erimek</t>
+  </si>
+  <si>
+    <t>meltem</t>
+  </si>
+  <si>
+    <t>Meltem esti, dondurma eridi</t>
+  </si>
+  <si>
+    <t>candy</t>
+  </si>
+  <si>
+    <t>kendi</t>
+  </si>
+  <si>
+    <t>Şekerlerin hepsini kendi yedi</t>
+  </si>
+  <si>
+    <t>cook</t>
+  </si>
+  <si>
+    <t>yemek pişirmek</t>
+  </si>
+  <si>
+    <t>kuku</t>
+  </si>
+  <si>
+    <t>Kuku kuşu yemek pişirdi</t>
+  </si>
+  <si>
+    <t>middle</t>
+  </si>
+  <si>
+    <t>orta</t>
+  </si>
+  <si>
+    <t>midye</t>
+  </si>
+  <si>
+    <t>Midyeyi tam ortadan böldü</t>
+  </si>
+  <si>
+    <t>shell</t>
+  </si>
+  <si>
+    <t>kabuk</t>
+  </si>
+  <si>
+    <t>şelale</t>
+  </si>
+  <si>
+    <t>Şelaleden kabuklar döküldü</t>
+  </si>
+  <si>
+    <t>hunt</t>
+  </si>
+  <si>
+    <t>avlamak</t>
+  </si>
+  <si>
+    <t>hantal</t>
+  </si>
+  <si>
+    <t>Hantal avcı avı kaçırdı</t>
+  </si>
+  <si>
+    <t>dinner</t>
+  </si>
+  <si>
+    <t>akşam yemeği</t>
+  </si>
+  <si>
+    <t>dinar</t>
+  </si>
+  <si>
+    <t>Akşam yemeğini dinarla ödedi</t>
+  </si>
+  <si>
+    <t>prize</t>
+  </si>
+  <si>
+    <t>ödül</t>
+  </si>
+  <si>
+    <t>priz</t>
+  </si>
+  <si>
+    <t>Ödülü prize taktı</t>
+  </si>
+  <si>
+    <t>wallet</t>
+  </si>
+  <si>
+    <t>cüzdan</t>
+  </si>
+  <si>
+    <t>valla</t>
+  </si>
+  <si>
+    <t>Valla cüzdanım boş!</t>
+  </si>
+  <si>
+    <t>fog</t>
+  </si>
+  <si>
+    <t>fok</t>
+  </si>
+  <si>
+    <t>Fok sisin içinde kayboldu</t>
+  </si>
+  <si>
+    <t>port</t>
+  </si>
+  <si>
+    <t>liman</t>
+  </si>
+  <si>
+    <t>portakal</t>
+  </si>
+  <si>
+    <t>Limana portakal gemisi yanaştı</t>
+  </si>
+  <si>
+    <t>sailor</t>
+  </si>
+  <si>
+    <t>denizci</t>
+  </si>
+  <si>
+    <t>seyyar</t>
+  </si>
+  <si>
+    <t>Seyyar satıcı denizciye simit sattı</t>
+  </si>
+  <si>
+    <t>ghost</t>
+  </si>
+  <si>
+    <t>hayalet</t>
+  </si>
+  <si>
+    <t>göster</t>
+  </si>
+  <si>
+    <t>Hayaleti göster!</t>
+  </si>
+  <si>
+    <t>luck</t>
+  </si>
+  <si>
+    <t>şans</t>
+  </si>
+  <si>
+    <t>lak lak</t>
+  </si>
+  <si>
+    <t>Lak lak ederken şansını kaçırdı</t>
+  </si>
+  <si>
+    <t>trap</t>
+  </si>
+  <si>
+    <t>tuzak</t>
+  </si>
+  <si>
+    <t>tırpan</t>
+  </si>
+  <si>
+    <t>Tuzağı tırpanla kesti</t>
+  </si>
+  <si>
+    <t>cliff</t>
+  </si>
+  <si>
+    <t>uçurum</t>
+  </si>
+  <si>
+    <t>kılıf</t>
+  </si>
+  <si>
+    <t>Uçuruma kılıf geçirmişler</t>
+  </si>
+  <si>
+    <t>hay</t>
+  </si>
+  <si>
+    <t>saman</t>
+  </si>
+  <si>
+    <t>hey</t>
+  </si>
+  <si>
+    <t>Hey, saman yanıyor!</t>
+  </si>
+  <si>
+    <t>bubble</t>
+  </si>
+  <si>
+    <t>baloncuk</t>
+  </si>
+  <si>
+    <t>baba</t>
+  </si>
+  <si>
+    <t>Baba baloncuk üfledi</t>
+  </si>
+  <si>
+    <t>climb</t>
+  </si>
+  <si>
+    <t>tırmanmak</t>
+  </si>
+  <si>
+    <t>klima</t>
+  </si>
+  <si>
+    <t>Klimaya tırmandı</t>
+  </si>
+  <si>
+    <t>pray</t>
+  </si>
+  <si>
+    <t>dua etmek</t>
+  </si>
+  <si>
+    <t>pire</t>
+  </si>
+  <si>
+    <t>Dua ederken pire ısırdı</t>
+  </si>
+  <si>
+    <t>beg</t>
+  </si>
+  <si>
+    <t>yalvarmak</t>
+  </si>
+  <si>
+    <t>bey</t>
+  </si>
+  <si>
+    <t>Bey, uşağına yalvardı</t>
+  </si>
+  <si>
+    <t>rob</t>
+  </si>
+  <si>
+    <t>robot</t>
+  </si>
+  <si>
+    <t>Robot bankayı soydu</t>
+  </si>
+  <si>
+    <t>rough</t>
+  </si>
+  <si>
+    <t>pürüzlü</t>
+  </si>
+  <si>
+    <t>raf</t>
+  </si>
+  <si>
+    <t>Raf öyle pürüzlü ki kazağım takıldı</t>
+  </si>
+  <si>
+    <t>deaf</t>
+  </si>
+  <si>
+    <t>sağır</t>
+  </si>
+  <si>
+    <t>def</t>
+  </si>
+  <si>
+    <t>Sağır adam def çalıyor</t>
+  </si>
+  <si>
+    <t>crowd</t>
+  </si>
+  <si>
+    <t>kalabalık</t>
+  </si>
+  <si>
+    <t>kravat</t>
+  </si>
+  <si>
+    <t>Kalabalığın hepsi kravatlı</t>
+  </si>
+  <si>
+    <t>page</t>
+  </si>
+  <si>
+    <t>sayfa</t>
+  </si>
+  <si>
+    <t>peçe</t>
+  </si>
+  <si>
+    <t>Sayfaya peçe örttü</t>
+  </si>
+  <si>
+    <t>cherry</t>
+  </si>
+  <si>
+    <t>kiraz</t>
+  </si>
+  <si>
+    <t>yeniçeri</t>
+  </si>
+  <si>
+    <t>Yeniçeri kiraz yedi</t>
+  </si>
+  <si>
+    <t>KART HAVUZU — 400 KART</t>
   </si>
   <si>
     <t>Zorluk: Kolay = ilk 1000 kelime · Orta = günlük ama daha seyrek · Zor = ileri seviye veya niş</t>
@@ -4567,7 +5743,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I301"/>
+  <dimension ref="A1:I401"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -12708,6 +13884,2906 @@
         <v>1386</v>
       </c>
       <c r="I301" s="7"/>
+    </row>
+    <row r="302" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A302">
+        <v>301</v>
+      </c>
+      <c r="B302" t="s">
+        <v>1387</v>
+      </c>
+      <c r="C302" t="s">
+        <v>1388</v>
+      </c>
+      <c r="D302" t="s">
+        <v>11</v>
+      </c>
+      <c r="E302" t="s">
+        <v>1389</v>
+      </c>
+      <c r="F302" t="s">
+        <v>1390</v>
+      </c>
+      <c r="G302" t="s">
+        <v>13</v>
+      </c>
+      <c r="H302" t="s">
+        <v>1390</v>
+      </c>
+      <c r="I302" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="303" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A303">
+        <v>302</v>
+      </c>
+      <c r="B303" t="s">
+        <v>1392</v>
+      </c>
+      <c r="C303" t="s">
+        <v>1393</v>
+      </c>
+      <c r="D303" t="s">
+        <v>11</v>
+      </c>
+      <c r="E303" t="s">
+        <v>1394</v>
+      </c>
+      <c r="F303" t="s">
+        <v>1395</v>
+      </c>
+      <c r="G303" t="s">
+        <v>13</v>
+      </c>
+      <c r="H303" t="s">
+        <v>1395</v>
+      </c>
+      <c r="I303" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="304" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A304">
+        <v>303</v>
+      </c>
+      <c r="B304" t="s">
+        <v>1396</v>
+      </c>
+      <c r="C304" t="s">
+        <v>1397</v>
+      </c>
+      <c r="D304" t="s">
+        <v>11</v>
+      </c>
+      <c r="E304" t="s">
+        <v>1398</v>
+      </c>
+      <c r="F304" t="s">
+        <v>1399</v>
+      </c>
+      <c r="G304" t="s">
+        <v>13</v>
+      </c>
+      <c r="H304" t="s">
+        <v>1399</v>
+      </c>
+      <c r="I304" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="305" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A305">
+        <v>304</v>
+      </c>
+      <c r="B305" t="s">
+        <v>1400</v>
+      </c>
+      <c r="C305" t="s">
+        <v>1401</v>
+      </c>
+      <c r="D305" t="s">
+        <v>11</v>
+      </c>
+      <c r="E305" t="s">
+        <v>1402</v>
+      </c>
+      <c r="F305" t="s">
+        <v>1403</v>
+      </c>
+      <c r="G305" t="s">
+        <v>13</v>
+      </c>
+      <c r="H305" t="s">
+        <v>1403</v>
+      </c>
+      <c r="I305" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="306" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A306">
+        <v>305</v>
+      </c>
+      <c r="B306" t="s">
+        <v>1404</v>
+      </c>
+      <c r="C306" t="s">
+        <v>1405</v>
+      </c>
+      <c r="D306" t="s">
+        <v>11</v>
+      </c>
+      <c r="E306" t="s">
+        <v>1406</v>
+      </c>
+      <c r="F306" t="s">
+        <v>1407</v>
+      </c>
+      <c r="G306" t="s">
+        <v>13</v>
+      </c>
+      <c r="H306" t="s">
+        <v>1407</v>
+      </c>
+      <c r="I306" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="307" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A307">
+        <v>306</v>
+      </c>
+      <c r="B307" t="s">
+        <v>1408</v>
+      </c>
+      <c r="C307" t="s">
+        <v>1409</v>
+      </c>
+      <c r="D307" t="s">
+        <v>11</v>
+      </c>
+      <c r="E307" t="s">
+        <v>1410</v>
+      </c>
+      <c r="F307" t="s">
+        <v>1411</v>
+      </c>
+      <c r="G307" t="s">
+        <v>13</v>
+      </c>
+      <c r="H307" t="s">
+        <v>1411</v>
+      </c>
+      <c r="I307" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="308" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A308">
+        <v>307</v>
+      </c>
+      <c r="B308" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C308" t="s">
+        <v>1413</v>
+      </c>
+      <c r="D308" t="s">
+        <v>11</v>
+      </c>
+      <c r="E308" t="s">
+        <v>1414</v>
+      </c>
+      <c r="F308" t="s">
+        <v>1415</v>
+      </c>
+      <c r="G308" t="s">
+        <v>13</v>
+      </c>
+      <c r="H308" t="s">
+        <v>1415</v>
+      </c>
+      <c r="I308" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="309" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A309">
+        <v>308</v>
+      </c>
+      <c r="B309" t="s">
+        <v>1416</v>
+      </c>
+      <c r="C309" t="s">
+        <v>1417</v>
+      </c>
+      <c r="D309" t="s">
+        <v>11</v>
+      </c>
+      <c r="E309" t="s">
+        <v>1418</v>
+      </c>
+      <c r="F309" t="s">
+        <v>1419</v>
+      </c>
+      <c r="G309" t="s">
+        <v>13</v>
+      </c>
+      <c r="H309" t="s">
+        <v>1419</v>
+      </c>
+      <c r="I309" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="310" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A310">
+        <v>309</v>
+      </c>
+      <c r="B310" t="s">
+        <v>1420</v>
+      </c>
+      <c r="C310" t="s">
+        <v>1421</v>
+      </c>
+      <c r="D310" t="s">
+        <v>11</v>
+      </c>
+      <c r="E310" t="s">
+        <v>1422</v>
+      </c>
+      <c r="F310" t="s">
+        <v>1423</v>
+      </c>
+      <c r="G310" t="s">
+        <v>487</v>
+      </c>
+      <c r="H310" t="s">
+        <v>1423</v>
+      </c>
+      <c r="I310" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="311" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A311">
+        <v>310</v>
+      </c>
+      <c r="B311" t="s">
+        <v>1424</v>
+      </c>
+      <c r="C311" t="s">
+        <v>1425</v>
+      </c>
+      <c r="D311" t="s">
+        <v>11</v>
+      </c>
+      <c r="E311" t="s">
+        <v>1426</v>
+      </c>
+      <c r="F311" t="s">
+        <v>1427</v>
+      </c>
+      <c r="G311" t="s">
+        <v>487</v>
+      </c>
+      <c r="H311" t="s">
+        <v>1427</v>
+      </c>
+      <c r="I311" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="312" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A312">
+        <v>311</v>
+      </c>
+      <c r="B312" t="s">
+        <v>1428</v>
+      </c>
+      <c r="C312" t="s">
+        <v>1429</v>
+      </c>
+      <c r="D312" t="s">
+        <v>11</v>
+      </c>
+      <c r="E312" t="s">
+        <v>1430</v>
+      </c>
+      <c r="F312" t="s">
+        <v>1431</v>
+      </c>
+      <c r="G312" t="s">
+        <v>13</v>
+      </c>
+      <c r="H312" t="s">
+        <v>1431</v>
+      </c>
+      <c r="I312" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="313" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A313">
+        <v>312</v>
+      </c>
+      <c r="B313" t="s">
+        <v>1432</v>
+      </c>
+      <c r="C313" t="s">
+        <v>1433</v>
+      </c>
+      <c r="D313" t="s">
+        <v>11</v>
+      </c>
+      <c r="E313" t="s">
+        <v>1434</v>
+      </c>
+      <c r="F313" t="s">
+        <v>1435</v>
+      </c>
+      <c r="G313" t="s">
+        <v>13</v>
+      </c>
+      <c r="H313" t="s">
+        <v>1435</v>
+      </c>
+      <c r="I313" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="314" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A314">
+        <v>313</v>
+      </c>
+      <c r="B314" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C314" t="s">
+        <v>1437</v>
+      </c>
+      <c r="D314" t="s">
+        <v>11</v>
+      </c>
+      <c r="E314" t="s">
+        <v>1438</v>
+      </c>
+      <c r="F314" t="s">
+        <v>1439</v>
+      </c>
+      <c r="G314" t="s">
+        <v>13</v>
+      </c>
+      <c r="H314" t="s">
+        <v>1439</v>
+      </c>
+      <c r="I314" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="315" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A315">
+        <v>314</v>
+      </c>
+      <c r="B315" t="s">
+        <v>1440</v>
+      </c>
+      <c r="C315" t="s">
+        <v>1441</v>
+      </c>
+      <c r="D315" t="s">
+        <v>11</v>
+      </c>
+      <c r="E315" t="s">
+        <v>1442</v>
+      </c>
+      <c r="F315" t="s">
+        <v>1443</v>
+      </c>
+      <c r="G315" t="s">
+        <v>13</v>
+      </c>
+      <c r="H315" t="s">
+        <v>1443</v>
+      </c>
+      <c r="I315" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="316" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A316">
+        <v>315</v>
+      </c>
+      <c r="B316" t="s">
+        <v>1444</v>
+      </c>
+      <c r="C316" t="s">
+        <v>1445</v>
+      </c>
+      <c r="D316" t="s">
+        <v>11</v>
+      </c>
+      <c r="E316" t="s">
+        <v>1446</v>
+      </c>
+      <c r="F316" t="s">
+        <v>1447</v>
+      </c>
+      <c r="G316" t="s">
+        <v>487</v>
+      </c>
+      <c r="H316" t="s">
+        <v>1447</v>
+      </c>
+      <c r="I316" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="317" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A317">
+        <v>316</v>
+      </c>
+      <c r="B317" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C317" t="s">
+        <v>1449</v>
+      </c>
+      <c r="D317" t="s">
+        <v>11</v>
+      </c>
+      <c r="E317" t="s">
+        <v>1450</v>
+      </c>
+      <c r="F317" t="s">
+        <v>1451</v>
+      </c>
+      <c r="G317" t="s">
+        <v>13</v>
+      </c>
+      <c r="H317" t="s">
+        <v>1451</v>
+      </c>
+      <c r="I317" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="318" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A318">
+        <v>317</v>
+      </c>
+      <c r="B318" t="s">
+        <v>1452</v>
+      </c>
+      <c r="C318" t="s">
+        <v>1453</v>
+      </c>
+      <c r="D318" t="s">
+        <v>11</v>
+      </c>
+      <c r="E318" t="s">
+        <v>1454</v>
+      </c>
+      <c r="F318" t="s">
+        <v>1455</v>
+      </c>
+      <c r="G318" t="s">
+        <v>487</v>
+      </c>
+      <c r="H318" t="s">
+        <v>1455</v>
+      </c>
+      <c r="I318" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="319" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A319">
+        <v>318</v>
+      </c>
+      <c r="B319" t="s">
+        <v>1456</v>
+      </c>
+      <c r="C319" t="s">
+        <v>1457</v>
+      </c>
+      <c r="D319" t="s">
+        <v>11</v>
+      </c>
+      <c r="E319" t="s">
+        <v>1458</v>
+      </c>
+      <c r="F319" t="s">
+        <v>1459</v>
+      </c>
+      <c r="G319" t="s">
+        <v>13</v>
+      </c>
+      <c r="H319" t="s">
+        <v>1459</v>
+      </c>
+      <c r="I319" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="320" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A320">
+        <v>319</v>
+      </c>
+      <c r="B320" t="s">
+        <v>1460</v>
+      </c>
+      <c r="C320" t="s">
+        <v>1461</v>
+      </c>
+      <c r="D320" t="s">
+        <v>11</v>
+      </c>
+      <c r="E320" t="s">
+        <v>1462</v>
+      </c>
+      <c r="F320" t="s">
+        <v>1463</v>
+      </c>
+      <c r="G320" t="s">
+        <v>13</v>
+      </c>
+      <c r="H320" t="s">
+        <v>1463</v>
+      </c>
+      <c r="I320" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="321" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A321">
+        <v>320</v>
+      </c>
+      <c r="B321" t="s">
+        <v>1464</v>
+      </c>
+      <c r="C321" t="s">
+        <v>1465</v>
+      </c>
+      <c r="D321" t="s">
+        <v>11</v>
+      </c>
+      <c r="E321" t="s">
+        <v>1464</v>
+      </c>
+      <c r="F321" t="s">
+        <v>1466</v>
+      </c>
+      <c r="G321" t="s">
+        <v>13</v>
+      </c>
+      <c r="H321" t="s">
+        <v>1466</v>
+      </c>
+      <c r="I321" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="322" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A322">
+        <v>321</v>
+      </c>
+      <c r="B322" t="s">
+        <v>1467</v>
+      </c>
+      <c r="C322" t="s">
+        <v>1468</v>
+      </c>
+      <c r="D322" t="s">
+        <v>11</v>
+      </c>
+      <c r="E322" t="s">
+        <v>1469</v>
+      </c>
+      <c r="F322" t="s">
+        <v>1470</v>
+      </c>
+      <c r="G322" t="s">
+        <v>13</v>
+      </c>
+      <c r="H322" t="s">
+        <v>1470</v>
+      </c>
+      <c r="I322" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="323" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A323">
+        <v>322</v>
+      </c>
+      <c r="B323" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C323" t="s">
+        <v>1472</v>
+      </c>
+      <c r="D323" t="s">
+        <v>11</v>
+      </c>
+      <c r="E323" t="s">
+        <v>1473</v>
+      </c>
+      <c r="F323" t="s">
+        <v>1474</v>
+      </c>
+      <c r="G323" t="s">
+        <v>13</v>
+      </c>
+      <c r="H323" t="s">
+        <v>1474</v>
+      </c>
+      <c r="I323" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="324" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A324">
+        <v>323</v>
+      </c>
+      <c r="B324" t="s">
+        <v>1475</v>
+      </c>
+      <c r="C324" t="s">
+        <v>1476</v>
+      </c>
+      <c r="D324" t="s">
+        <v>11</v>
+      </c>
+      <c r="E324" t="s">
+        <v>1477</v>
+      </c>
+      <c r="F324" t="s">
+        <v>1478</v>
+      </c>
+      <c r="G324" t="s">
+        <v>13</v>
+      </c>
+      <c r="H324" t="s">
+        <v>1478</v>
+      </c>
+      <c r="I324" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="325" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A325">
+        <v>324</v>
+      </c>
+      <c r="B325" t="s">
+        <v>1479</v>
+      </c>
+      <c r="C325" t="s">
+        <v>1480</v>
+      </c>
+      <c r="D325" t="s">
+        <v>11</v>
+      </c>
+      <c r="E325" t="s">
+        <v>1481</v>
+      </c>
+      <c r="F325" t="s">
+        <v>1482</v>
+      </c>
+      <c r="G325" t="s">
+        <v>487</v>
+      </c>
+      <c r="H325" t="s">
+        <v>1482</v>
+      </c>
+      <c r="I325" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="326" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A326">
+        <v>325</v>
+      </c>
+      <c r="B326" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C326" t="s">
+        <v>1484</v>
+      </c>
+      <c r="D326" t="s">
+        <v>11</v>
+      </c>
+      <c r="E326" t="s">
+        <v>1485</v>
+      </c>
+      <c r="F326" t="s">
+        <v>1486</v>
+      </c>
+      <c r="G326" t="s">
+        <v>13</v>
+      </c>
+      <c r="H326" t="s">
+        <v>1486</v>
+      </c>
+      <c r="I326" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="327" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A327">
+        <v>326</v>
+      </c>
+      <c r="B327" t="s">
+        <v>1487</v>
+      </c>
+      <c r="C327" t="s">
+        <v>1488</v>
+      </c>
+      <c r="D327" t="s">
+        <v>11</v>
+      </c>
+      <c r="E327" t="s">
+        <v>1489</v>
+      </c>
+      <c r="F327" t="s">
+        <v>1490</v>
+      </c>
+      <c r="G327" t="s">
+        <v>13</v>
+      </c>
+      <c r="H327" t="s">
+        <v>1490</v>
+      </c>
+      <c r="I327" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="328" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A328">
+        <v>327</v>
+      </c>
+      <c r="B328" t="s">
+        <v>1491</v>
+      </c>
+      <c r="C328" t="s">
+        <v>1492</v>
+      </c>
+      <c r="D328" t="s">
+        <v>11</v>
+      </c>
+      <c r="E328" t="s">
+        <v>1493</v>
+      </c>
+      <c r="F328" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G328" t="s">
+        <v>487</v>
+      </c>
+      <c r="H328" t="s">
+        <v>1494</v>
+      </c>
+      <c r="I328" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="329" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A329">
+        <v>328</v>
+      </c>
+      <c r="B329" t="s">
+        <v>1495</v>
+      </c>
+      <c r="C329" t="s">
+        <v>1496</v>
+      </c>
+      <c r="D329" t="s">
+        <v>11</v>
+      </c>
+      <c r="E329" t="s">
+        <v>1497</v>
+      </c>
+      <c r="F329" t="s">
+        <v>1498</v>
+      </c>
+      <c r="G329" t="s">
+        <v>13</v>
+      </c>
+      <c r="H329" t="s">
+        <v>1498</v>
+      </c>
+      <c r="I329" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="330" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A330">
+        <v>329</v>
+      </c>
+      <c r="B330" t="s">
+        <v>1499</v>
+      </c>
+      <c r="C330" t="s">
+        <v>1500</v>
+      </c>
+      <c r="D330" t="s">
+        <v>11</v>
+      </c>
+      <c r="E330" t="s">
+        <v>1501</v>
+      </c>
+      <c r="F330" t="s">
+        <v>1502</v>
+      </c>
+      <c r="G330" t="s">
+        <v>13</v>
+      </c>
+      <c r="H330" t="s">
+        <v>1502</v>
+      </c>
+      <c r="I330" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="331" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A331">
+        <v>330</v>
+      </c>
+      <c r="B331" t="s">
+        <v>1503</v>
+      </c>
+      <c r="C331" t="s">
+        <v>1504</v>
+      </c>
+      <c r="D331" t="s">
+        <v>11</v>
+      </c>
+      <c r="E331" t="s">
+        <v>1505</v>
+      </c>
+      <c r="F331" t="s">
+        <v>1506</v>
+      </c>
+      <c r="G331" t="s">
+        <v>13</v>
+      </c>
+      <c r="H331" t="s">
+        <v>1506</v>
+      </c>
+      <c r="I331" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="332" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A332">
+        <v>331</v>
+      </c>
+      <c r="B332" t="s">
+        <v>1507</v>
+      </c>
+      <c r="C332" t="s">
+        <v>1508</v>
+      </c>
+      <c r="D332" t="s">
+        <v>11</v>
+      </c>
+      <c r="E332" t="s">
+        <v>1509</v>
+      </c>
+      <c r="F332" t="s">
+        <v>1510</v>
+      </c>
+      <c r="G332" t="s">
+        <v>13</v>
+      </c>
+      <c r="H332" t="s">
+        <v>1510</v>
+      </c>
+      <c r="I332" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="333" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A333">
+        <v>332</v>
+      </c>
+      <c r="B333" t="s">
+        <v>1511</v>
+      </c>
+      <c r="C333" t="s">
+        <v>1512</v>
+      </c>
+      <c r="D333" t="s">
+        <v>11</v>
+      </c>
+      <c r="E333" t="s">
+        <v>1513</v>
+      </c>
+      <c r="F333" t="s">
+        <v>1514</v>
+      </c>
+      <c r="G333" t="s">
+        <v>13</v>
+      </c>
+      <c r="H333" t="s">
+        <v>1514</v>
+      </c>
+      <c r="I333" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="334" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A334">
+        <v>333</v>
+      </c>
+      <c r="B334" t="s">
+        <v>1515</v>
+      </c>
+      <c r="C334" t="s">
+        <v>1516</v>
+      </c>
+      <c r="D334" t="s">
+        <v>11</v>
+      </c>
+      <c r="E334" t="s">
+        <v>1517</v>
+      </c>
+      <c r="F334" t="s">
+        <v>1518</v>
+      </c>
+      <c r="G334" t="s">
+        <v>13</v>
+      </c>
+      <c r="H334" t="s">
+        <v>1518</v>
+      </c>
+      <c r="I334" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="335" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A335">
+        <v>334</v>
+      </c>
+      <c r="B335" t="s">
+        <v>1519</v>
+      </c>
+      <c r="C335" t="s">
+        <v>1520</v>
+      </c>
+      <c r="D335" t="s">
+        <v>11</v>
+      </c>
+      <c r="E335" t="s">
+        <v>1521</v>
+      </c>
+      <c r="F335" t="s">
+        <v>1522</v>
+      </c>
+      <c r="G335" t="s">
+        <v>13</v>
+      </c>
+      <c r="H335" t="s">
+        <v>1522</v>
+      </c>
+      <c r="I335" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="336" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A336">
+        <v>335</v>
+      </c>
+      <c r="B336" t="s">
+        <v>1523</v>
+      </c>
+      <c r="C336" t="s">
+        <v>1524</v>
+      </c>
+      <c r="D336" t="s">
+        <v>11</v>
+      </c>
+      <c r="E336" t="s">
+        <v>1525</v>
+      </c>
+      <c r="F336" t="s">
+        <v>1526</v>
+      </c>
+      <c r="G336" t="s">
+        <v>13</v>
+      </c>
+      <c r="H336" t="s">
+        <v>1526</v>
+      </c>
+      <c r="I336" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="337" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A337">
+        <v>336</v>
+      </c>
+      <c r="B337" t="s">
+        <v>1527</v>
+      </c>
+      <c r="C337" t="s">
+        <v>1528</v>
+      </c>
+      <c r="D337" t="s">
+        <v>11</v>
+      </c>
+      <c r="E337" t="s">
+        <v>1529</v>
+      </c>
+      <c r="F337" t="s">
+        <v>1530</v>
+      </c>
+      <c r="G337" t="s">
+        <v>487</v>
+      </c>
+      <c r="H337" t="s">
+        <v>1530</v>
+      </c>
+      <c r="I337" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="338" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A338">
+        <v>337</v>
+      </c>
+      <c r="B338" t="s">
+        <v>1531</v>
+      </c>
+      <c r="C338" t="s">
+        <v>1532</v>
+      </c>
+      <c r="D338" t="s">
+        <v>32</v>
+      </c>
+      <c r="E338" t="s">
+        <v>1533</v>
+      </c>
+      <c r="F338" t="s">
+        <v>1534</v>
+      </c>
+      <c r="G338" t="s">
+        <v>487</v>
+      </c>
+      <c r="H338" t="s">
+        <v>1534</v>
+      </c>
+      <c r="I338" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="339" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A339">
+        <v>338</v>
+      </c>
+      <c r="B339" t="s">
+        <v>1535</v>
+      </c>
+      <c r="C339" t="s">
+        <v>1536</v>
+      </c>
+      <c r="D339" t="s">
+        <v>32</v>
+      </c>
+      <c r="E339" t="s">
+        <v>1537</v>
+      </c>
+      <c r="F339" t="s">
+        <v>1538</v>
+      </c>
+      <c r="G339" t="s">
+        <v>13</v>
+      </c>
+      <c r="H339" t="s">
+        <v>1538</v>
+      </c>
+      <c r="I339" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="340" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A340">
+        <v>339</v>
+      </c>
+      <c r="B340" t="s">
+        <v>1539</v>
+      </c>
+      <c r="C340" t="s">
+        <v>1540</v>
+      </c>
+      <c r="D340" t="s">
+        <v>11</v>
+      </c>
+      <c r="E340" t="s">
+        <v>1541</v>
+      </c>
+      <c r="F340" t="s">
+        <v>1542</v>
+      </c>
+      <c r="G340" t="s">
+        <v>487</v>
+      </c>
+      <c r="H340" t="s">
+        <v>1542</v>
+      </c>
+      <c r="I340" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="341" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A341">
+        <v>340</v>
+      </c>
+      <c r="B341" t="s">
+        <v>1543</v>
+      </c>
+      <c r="C341" t="s">
+        <v>1544</v>
+      </c>
+      <c r="D341" t="s">
+        <v>11</v>
+      </c>
+      <c r="E341" t="s">
+        <v>1545</v>
+      </c>
+      <c r="F341" t="s">
+        <v>1546</v>
+      </c>
+      <c r="G341" t="s">
+        <v>13</v>
+      </c>
+      <c r="H341" t="s">
+        <v>1546</v>
+      </c>
+      <c r="I341" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="342" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A342">
+        <v>341</v>
+      </c>
+      <c r="B342" t="s">
+        <v>1547</v>
+      </c>
+      <c r="C342" t="s">
+        <v>1548</v>
+      </c>
+      <c r="D342" t="s">
+        <v>11</v>
+      </c>
+      <c r="E342" t="s">
+        <v>1549</v>
+      </c>
+      <c r="F342" t="s">
+        <v>1550</v>
+      </c>
+      <c r="G342" t="s">
+        <v>13</v>
+      </c>
+      <c r="H342" t="s">
+        <v>1550</v>
+      </c>
+      <c r="I342" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="343" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A343">
+        <v>342</v>
+      </c>
+      <c r="B343" t="s">
+        <v>1551</v>
+      </c>
+      <c r="C343" t="s">
+        <v>1552</v>
+      </c>
+      <c r="D343" t="s">
+        <v>11</v>
+      </c>
+      <c r="E343" t="s">
+        <v>1553</v>
+      </c>
+      <c r="F343" t="s">
+        <v>1554</v>
+      </c>
+      <c r="G343" t="s">
+        <v>13</v>
+      </c>
+      <c r="H343" t="s">
+        <v>1554</v>
+      </c>
+      <c r="I343" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="344" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A344">
+        <v>343</v>
+      </c>
+      <c r="B344" t="s">
+        <v>1555</v>
+      </c>
+      <c r="C344" t="s">
+        <v>1556</v>
+      </c>
+      <c r="D344" t="s">
+        <v>11</v>
+      </c>
+      <c r="E344" t="s">
+        <v>1557</v>
+      </c>
+      <c r="F344" t="s">
+        <v>1558</v>
+      </c>
+      <c r="G344" t="s">
+        <v>487</v>
+      </c>
+      <c r="H344" t="s">
+        <v>1558</v>
+      </c>
+      <c r="I344" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="345" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A345">
+        <v>344</v>
+      </c>
+      <c r="B345" t="s">
+        <v>1559</v>
+      </c>
+      <c r="C345" t="s">
+        <v>1560</v>
+      </c>
+      <c r="D345" t="s">
+        <v>11</v>
+      </c>
+      <c r="E345" t="s">
+        <v>1561</v>
+      </c>
+      <c r="F345" t="s">
+        <v>1562</v>
+      </c>
+      <c r="G345" t="s">
+        <v>487</v>
+      </c>
+      <c r="H345" t="s">
+        <v>1562</v>
+      </c>
+      <c r="I345" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="346" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A346">
+        <v>345</v>
+      </c>
+      <c r="B346" t="s">
+        <v>1563</v>
+      </c>
+      <c r="C346" t="s">
+        <v>1564</v>
+      </c>
+      <c r="D346" t="s">
+        <v>11</v>
+      </c>
+      <c r="E346" t="s">
+        <v>1565</v>
+      </c>
+      <c r="F346" t="s">
+        <v>1566</v>
+      </c>
+      <c r="G346" t="s">
+        <v>487</v>
+      </c>
+      <c r="H346" t="s">
+        <v>1566</v>
+      </c>
+      <c r="I346" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="347" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A347">
+        <v>346</v>
+      </c>
+      <c r="B347" t="s">
+        <v>1567</v>
+      </c>
+      <c r="C347" t="s">
+        <v>1568</v>
+      </c>
+      <c r="D347" t="s">
+        <v>11</v>
+      </c>
+      <c r="E347" t="s">
+        <v>1569</v>
+      </c>
+      <c r="F347" t="s">
+        <v>1570</v>
+      </c>
+      <c r="G347" t="s">
+        <v>487</v>
+      </c>
+      <c r="H347" t="s">
+        <v>1570</v>
+      </c>
+      <c r="I347" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="348" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A348">
+        <v>347</v>
+      </c>
+      <c r="B348" t="s">
+        <v>1571</v>
+      </c>
+      <c r="C348" t="s">
+        <v>1572</v>
+      </c>
+      <c r="D348" t="s">
+        <v>11</v>
+      </c>
+      <c r="E348" t="s">
+        <v>1573</v>
+      </c>
+      <c r="F348" t="s">
+        <v>1574</v>
+      </c>
+      <c r="G348" t="s">
+        <v>487</v>
+      </c>
+      <c r="H348" t="s">
+        <v>1574</v>
+      </c>
+      <c r="I348" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="349" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A349">
+        <v>348</v>
+      </c>
+      <c r="B349" t="s">
+        <v>1575</v>
+      </c>
+      <c r="C349" t="s">
+        <v>1576</v>
+      </c>
+      <c r="D349" t="s">
+        <v>11</v>
+      </c>
+      <c r="E349" t="s">
+        <v>1577</v>
+      </c>
+      <c r="F349" t="s">
+        <v>1578</v>
+      </c>
+      <c r="G349" t="s">
+        <v>13</v>
+      </c>
+      <c r="H349" t="s">
+        <v>1578</v>
+      </c>
+      <c r="I349" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="350" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A350">
+        <v>349</v>
+      </c>
+      <c r="B350" t="s">
+        <v>1579</v>
+      </c>
+      <c r="C350" t="s">
+        <v>1580</v>
+      </c>
+      <c r="D350" t="s">
+        <v>11</v>
+      </c>
+      <c r="E350" t="s">
+        <v>1579</v>
+      </c>
+      <c r="F350" t="s">
+        <v>1581</v>
+      </c>
+      <c r="G350" t="s">
+        <v>13</v>
+      </c>
+      <c r="H350" t="s">
+        <v>1581</v>
+      </c>
+      <c r="I350" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="351" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A351">
+        <v>350</v>
+      </c>
+      <c r="B351" t="s">
+        <v>1582</v>
+      </c>
+      <c r="C351" t="s">
+        <v>1583</v>
+      </c>
+      <c r="D351" t="s">
+        <v>32</v>
+      </c>
+      <c r="E351" t="s">
+        <v>1584</v>
+      </c>
+      <c r="F351" t="s">
+        <v>1585</v>
+      </c>
+      <c r="G351" t="s">
+        <v>13</v>
+      </c>
+      <c r="H351" t="s">
+        <v>1585</v>
+      </c>
+      <c r="I351" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="352" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A352">
+        <v>351</v>
+      </c>
+      <c r="B352" t="s">
+        <v>1586</v>
+      </c>
+      <c r="C352" t="s">
+        <v>784</v>
+      </c>
+      <c r="D352" t="s">
+        <v>11</v>
+      </c>
+      <c r="E352" t="s">
+        <v>1587</v>
+      </c>
+      <c r="F352" t="s">
+        <v>1588</v>
+      </c>
+      <c r="G352" t="s">
+        <v>13</v>
+      </c>
+      <c r="H352" t="s">
+        <v>1588</v>
+      </c>
+      <c r="I352" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="353" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A353">
+        <v>352</v>
+      </c>
+      <c r="B353" t="s">
+        <v>1589</v>
+      </c>
+      <c r="C353" t="s">
+        <v>1590</v>
+      </c>
+      <c r="D353" t="s">
+        <v>11</v>
+      </c>
+      <c r="E353" t="s">
+        <v>1591</v>
+      </c>
+      <c r="F353" t="s">
+        <v>1592</v>
+      </c>
+      <c r="G353" t="s">
+        <v>487</v>
+      </c>
+      <c r="H353" t="s">
+        <v>1592</v>
+      </c>
+      <c r="I353" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="354" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A354">
+        <v>353</v>
+      </c>
+      <c r="B354" t="s">
+        <v>1593</v>
+      </c>
+      <c r="C354" t="s">
+        <v>1594</v>
+      </c>
+      <c r="D354" t="s">
+        <v>11</v>
+      </c>
+      <c r="E354" t="s">
+        <v>1595</v>
+      </c>
+      <c r="F354" t="s">
+        <v>1596</v>
+      </c>
+      <c r="G354" t="s">
+        <v>13</v>
+      </c>
+      <c r="H354" t="s">
+        <v>1596</v>
+      </c>
+      <c r="I354" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="355" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A355">
+        <v>354</v>
+      </c>
+      <c r="B355" t="s">
+        <v>1597</v>
+      </c>
+      <c r="C355" t="s">
+        <v>1598</v>
+      </c>
+      <c r="D355" t="s">
+        <v>11</v>
+      </c>
+      <c r="E355" t="s">
+        <v>1599</v>
+      </c>
+      <c r="F355" t="s">
+        <v>1600</v>
+      </c>
+      <c r="G355" t="s">
+        <v>13</v>
+      </c>
+      <c r="H355" t="s">
+        <v>1600</v>
+      </c>
+      <c r="I355" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="356" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A356">
+        <v>355</v>
+      </c>
+      <c r="B356" t="s">
+        <v>1601</v>
+      </c>
+      <c r="C356" t="s">
+        <v>1602</v>
+      </c>
+      <c r="D356" t="s">
+        <v>11</v>
+      </c>
+      <c r="E356" t="s">
+        <v>1603</v>
+      </c>
+      <c r="F356" t="s">
+        <v>1604</v>
+      </c>
+      <c r="G356" t="s">
+        <v>13</v>
+      </c>
+      <c r="H356" t="s">
+        <v>1604</v>
+      </c>
+      <c r="I356" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="357" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A357">
+        <v>356</v>
+      </c>
+      <c r="B357" t="s">
+        <v>1605</v>
+      </c>
+      <c r="C357" t="s">
+        <v>282</v>
+      </c>
+      <c r="D357" t="s">
+        <v>11</v>
+      </c>
+      <c r="E357" t="s">
+        <v>1606</v>
+      </c>
+      <c r="F357" t="s">
+        <v>1607</v>
+      </c>
+      <c r="G357" t="s">
+        <v>487</v>
+      </c>
+      <c r="H357" t="s">
+        <v>1607</v>
+      </c>
+      <c r="I357" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="358" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A358">
+        <v>357</v>
+      </c>
+      <c r="B358" t="s">
+        <v>1608</v>
+      </c>
+      <c r="C358" t="s">
+        <v>1609</v>
+      </c>
+      <c r="D358" t="s">
+        <v>11</v>
+      </c>
+      <c r="E358" t="s">
+        <v>1608</v>
+      </c>
+      <c r="F358" t="s">
+        <v>1610</v>
+      </c>
+      <c r="G358" t="s">
+        <v>487</v>
+      </c>
+      <c r="H358" t="s">
+        <v>1610</v>
+      </c>
+      <c r="I358" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="359" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A359">
+        <v>358</v>
+      </c>
+      <c r="B359" t="s">
+        <v>1611</v>
+      </c>
+      <c r="C359" t="s">
+        <v>1612</v>
+      </c>
+      <c r="D359" t="s">
+        <v>11</v>
+      </c>
+      <c r="E359" t="s">
+        <v>1613</v>
+      </c>
+      <c r="F359" t="s">
+        <v>1614</v>
+      </c>
+      <c r="G359" t="s">
+        <v>13</v>
+      </c>
+      <c r="H359" t="s">
+        <v>1614</v>
+      </c>
+      <c r="I359" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="360" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A360">
+        <v>359</v>
+      </c>
+      <c r="B360" t="s">
+        <v>1615</v>
+      </c>
+      <c r="C360" t="s">
+        <v>1616</v>
+      </c>
+      <c r="D360" t="s">
+        <v>11</v>
+      </c>
+      <c r="E360" t="s">
+        <v>1615</v>
+      </c>
+      <c r="F360" t="s">
+        <v>1617</v>
+      </c>
+      <c r="G360" t="s">
+        <v>487</v>
+      </c>
+      <c r="H360" t="s">
+        <v>1617</v>
+      </c>
+      <c r="I360" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="361" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A361">
+        <v>360</v>
+      </c>
+      <c r="B361" t="s">
+        <v>1618</v>
+      </c>
+      <c r="C361" t="s">
+        <v>1619</v>
+      </c>
+      <c r="D361" t="s">
+        <v>11</v>
+      </c>
+      <c r="E361" t="s">
+        <v>1620</v>
+      </c>
+      <c r="F361" t="s">
+        <v>1621</v>
+      </c>
+      <c r="G361" t="s">
+        <v>13</v>
+      </c>
+      <c r="H361" t="s">
+        <v>1621</v>
+      </c>
+      <c r="I361" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="362" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A362">
+        <v>361</v>
+      </c>
+      <c r="B362" t="s">
+        <v>1622</v>
+      </c>
+      <c r="C362" t="s">
+        <v>1623</v>
+      </c>
+      <c r="D362" t="s">
+        <v>11</v>
+      </c>
+      <c r="E362" t="s">
+        <v>1624</v>
+      </c>
+      <c r="F362" t="s">
+        <v>1625</v>
+      </c>
+      <c r="G362" t="s">
+        <v>13</v>
+      </c>
+      <c r="H362" t="s">
+        <v>1625</v>
+      </c>
+      <c r="I362" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="363" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A363">
+        <v>362</v>
+      </c>
+      <c r="B363" t="s">
+        <v>1626</v>
+      </c>
+      <c r="C363" t="s">
+        <v>1627</v>
+      </c>
+      <c r="D363" t="s">
+        <v>11</v>
+      </c>
+      <c r="E363" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F363" t="s">
+        <v>1629</v>
+      </c>
+      <c r="G363" t="s">
+        <v>13</v>
+      </c>
+      <c r="H363" t="s">
+        <v>1629</v>
+      </c>
+      <c r="I363" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="364" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A364">
+        <v>363</v>
+      </c>
+      <c r="B364" t="s">
+        <v>1630</v>
+      </c>
+      <c r="C364" t="s">
+        <v>1631</v>
+      </c>
+      <c r="D364" t="s">
+        <v>11</v>
+      </c>
+      <c r="E364" t="s">
+        <v>1632</v>
+      </c>
+      <c r="F364" t="s">
+        <v>1633</v>
+      </c>
+      <c r="G364" t="s">
+        <v>487</v>
+      </c>
+      <c r="H364" t="s">
+        <v>1633</v>
+      </c>
+      <c r="I364" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="365" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A365">
+        <v>364</v>
+      </c>
+      <c r="B365" t="s">
+        <v>1634</v>
+      </c>
+      <c r="C365" t="s">
+        <v>1635</v>
+      </c>
+      <c r="D365" t="s">
+        <v>11</v>
+      </c>
+      <c r="E365" t="s">
+        <v>1636</v>
+      </c>
+      <c r="F365" t="s">
+        <v>1637</v>
+      </c>
+      <c r="G365" t="s">
+        <v>13</v>
+      </c>
+      <c r="H365" t="s">
+        <v>1637</v>
+      </c>
+      <c r="I365" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="366" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A366">
+        <v>365</v>
+      </c>
+      <c r="B366" t="s">
+        <v>1638</v>
+      </c>
+      <c r="C366" t="s">
+        <v>1639</v>
+      </c>
+      <c r="D366" t="s">
+        <v>32</v>
+      </c>
+      <c r="E366" t="s">
+        <v>1640</v>
+      </c>
+      <c r="F366" t="s">
+        <v>1641</v>
+      </c>
+      <c r="G366" t="s">
+        <v>13</v>
+      </c>
+      <c r="H366" t="s">
+        <v>1641</v>
+      </c>
+      <c r="I366" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="367" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A367">
+        <v>366</v>
+      </c>
+      <c r="B367" t="s">
+        <v>1642</v>
+      </c>
+      <c r="C367" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D367" t="s">
+        <v>11</v>
+      </c>
+      <c r="E367" t="s">
+        <v>1644</v>
+      </c>
+      <c r="F367" t="s">
+        <v>1645</v>
+      </c>
+      <c r="G367" t="s">
+        <v>13</v>
+      </c>
+      <c r="H367" t="s">
+        <v>1645</v>
+      </c>
+      <c r="I367" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="368" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A368">
+        <v>367</v>
+      </c>
+      <c r="B368" t="s">
+        <v>1646</v>
+      </c>
+      <c r="C368" t="s">
+        <v>1647</v>
+      </c>
+      <c r="D368" t="s">
+        <v>11</v>
+      </c>
+      <c r="E368" t="s">
+        <v>1648</v>
+      </c>
+      <c r="F368" t="s">
+        <v>1649</v>
+      </c>
+      <c r="G368" t="s">
+        <v>13</v>
+      </c>
+      <c r="H368" t="s">
+        <v>1649</v>
+      </c>
+      <c r="I368" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="369" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A369">
+        <v>368</v>
+      </c>
+      <c r="B369" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C369" t="s">
+        <v>1651</v>
+      </c>
+      <c r="D369" t="s">
+        <v>32</v>
+      </c>
+      <c r="E369" t="s">
+        <v>1652</v>
+      </c>
+      <c r="F369" t="s">
+        <v>1653</v>
+      </c>
+      <c r="G369" t="s">
+        <v>13</v>
+      </c>
+      <c r="H369" t="s">
+        <v>1653</v>
+      </c>
+      <c r="I369" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="370" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A370">
+        <v>369</v>
+      </c>
+      <c r="B370" t="s">
+        <v>1654</v>
+      </c>
+      <c r="C370" t="s">
+        <v>1655</v>
+      </c>
+      <c r="D370" t="s">
+        <v>32</v>
+      </c>
+      <c r="E370" t="s">
+        <v>1656</v>
+      </c>
+      <c r="F370" t="s">
+        <v>1657</v>
+      </c>
+      <c r="G370" t="s">
+        <v>13</v>
+      </c>
+      <c r="H370" t="s">
+        <v>1657</v>
+      </c>
+      <c r="I370" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="371" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A371">
+        <v>370</v>
+      </c>
+      <c r="B371" t="s">
+        <v>1658</v>
+      </c>
+      <c r="C371" t="s">
+        <v>1659</v>
+      </c>
+      <c r="D371" t="s">
+        <v>32</v>
+      </c>
+      <c r="E371" t="s">
+        <v>1660</v>
+      </c>
+      <c r="F371" t="s">
+        <v>1661</v>
+      </c>
+      <c r="G371" t="s">
+        <v>13</v>
+      </c>
+      <c r="H371" t="s">
+        <v>1661</v>
+      </c>
+      <c r="I371" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="372" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A372">
+        <v>371</v>
+      </c>
+      <c r="B372" t="s">
+        <v>1662</v>
+      </c>
+      <c r="C372" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D372" t="s">
+        <v>11</v>
+      </c>
+      <c r="E372" t="s">
+        <v>1664</v>
+      </c>
+      <c r="F372" t="s">
+        <v>1665</v>
+      </c>
+      <c r="G372" t="s">
+        <v>13</v>
+      </c>
+      <c r="H372" t="s">
+        <v>1665</v>
+      </c>
+      <c r="I372" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="373" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A373">
+        <v>372</v>
+      </c>
+      <c r="B373" t="s">
+        <v>1666</v>
+      </c>
+      <c r="C373" t="s">
+        <v>1667</v>
+      </c>
+      <c r="D373" t="s">
+        <v>11</v>
+      </c>
+      <c r="E373" t="s">
+        <v>1668</v>
+      </c>
+      <c r="F373" t="s">
+        <v>1669</v>
+      </c>
+      <c r="G373" t="s">
+        <v>13</v>
+      </c>
+      <c r="H373" t="s">
+        <v>1669</v>
+      </c>
+      <c r="I373" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="374" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A374">
+        <v>373</v>
+      </c>
+      <c r="B374" t="s">
+        <v>1670</v>
+      </c>
+      <c r="C374" t="s">
+        <v>1671</v>
+      </c>
+      <c r="D374" t="s">
+        <v>11</v>
+      </c>
+      <c r="E374" t="s">
+        <v>1672</v>
+      </c>
+      <c r="F374" t="s">
+        <v>1673</v>
+      </c>
+      <c r="G374" t="s">
+        <v>13</v>
+      </c>
+      <c r="H374" t="s">
+        <v>1673</v>
+      </c>
+      <c r="I374" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="375" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A375">
+        <v>374</v>
+      </c>
+      <c r="B375" t="s">
+        <v>1674</v>
+      </c>
+      <c r="C375" t="s">
+        <v>1675</v>
+      </c>
+      <c r="D375" t="s">
+        <v>32</v>
+      </c>
+      <c r="E375" t="s">
+        <v>1676</v>
+      </c>
+      <c r="F375" t="s">
+        <v>1677</v>
+      </c>
+      <c r="G375" t="s">
+        <v>13</v>
+      </c>
+      <c r="H375" t="s">
+        <v>1677</v>
+      </c>
+      <c r="I375" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="376" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A376">
+        <v>375</v>
+      </c>
+      <c r="B376" t="s">
+        <v>1678</v>
+      </c>
+      <c r="C376" t="s">
+        <v>207</v>
+      </c>
+      <c r="D376" t="s">
+        <v>11</v>
+      </c>
+      <c r="E376" t="s">
+        <v>1679</v>
+      </c>
+      <c r="F376" t="s">
+        <v>1680</v>
+      </c>
+      <c r="G376" t="s">
+        <v>13</v>
+      </c>
+      <c r="H376" t="s">
+        <v>1680</v>
+      </c>
+      <c r="I376" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="377" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A377">
+        <v>376</v>
+      </c>
+      <c r="B377" t="s">
+        <v>1681</v>
+      </c>
+      <c r="C377" t="s">
+        <v>1682</v>
+      </c>
+      <c r="D377" t="s">
+        <v>11</v>
+      </c>
+      <c r="E377" t="s">
+        <v>1683</v>
+      </c>
+      <c r="F377" t="s">
+        <v>1684</v>
+      </c>
+      <c r="G377" t="s">
+        <v>487</v>
+      </c>
+      <c r="H377" t="s">
+        <v>1684</v>
+      </c>
+      <c r="I377" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="378" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A378">
+        <v>377</v>
+      </c>
+      <c r="B378" t="s">
+        <v>1685</v>
+      </c>
+      <c r="C378" t="s">
+        <v>1686</v>
+      </c>
+      <c r="D378" t="s">
+        <v>11</v>
+      </c>
+      <c r="E378" t="s">
+        <v>1687</v>
+      </c>
+      <c r="F378" t="s">
+        <v>1688</v>
+      </c>
+      <c r="G378" t="s">
+        <v>13</v>
+      </c>
+      <c r="H378" t="s">
+        <v>1688</v>
+      </c>
+      <c r="I378" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="379" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A379">
+        <v>378</v>
+      </c>
+      <c r="B379" t="s">
+        <v>1689</v>
+      </c>
+      <c r="C379" t="s">
+        <v>1690</v>
+      </c>
+      <c r="D379" t="s">
+        <v>32</v>
+      </c>
+      <c r="E379" t="s">
+        <v>1691</v>
+      </c>
+      <c r="F379" t="s">
+        <v>1692</v>
+      </c>
+      <c r="G379" t="s">
+        <v>487</v>
+      </c>
+      <c r="H379" t="s">
+        <v>1692</v>
+      </c>
+      <c r="I379" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="380" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A380">
+        <v>379</v>
+      </c>
+      <c r="B380" t="s">
+        <v>1693</v>
+      </c>
+      <c r="C380" t="s">
+        <v>1694</v>
+      </c>
+      <c r="D380" t="s">
+        <v>32</v>
+      </c>
+      <c r="E380" t="s">
+        <v>1695</v>
+      </c>
+      <c r="F380" t="s">
+        <v>1696</v>
+      </c>
+      <c r="G380" t="s">
+        <v>13</v>
+      </c>
+      <c r="H380" t="s">
+        <v>1696</v>
+      </c>
+      <c r="I380" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="381" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A381">
+        <v>380</v>
+      </c>
+      <c r="B381" t="s">
+        <v>1697</v>
+      </c>
+      <c r="C381" t="s">
+        <v>1698</v>
+      </c>
+      <c r="D381" t="s">
+        <v>11</v>
+      </c>
+      <c r="E381" t="s">
+        <v>1699</v>
+      </c>
+      <c r="F381" t="s">
+        <v>1700</v>
+      </c>
+      <c r="G381" t="s">
+        <v>13</v>
+      </c>
+      <c r="H381" t="s">
+        <v>1700</v>
+      </c>
+      <c r="I381" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="382" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A382">
+        <v>381</v>
+      </c>
+      <c r="B382" t="s">
+        <v>1701</v>
+      </c>
+      <c r="C382" t="s">
+        <v>1702</v>
+      </c>
+      <c r="D382" t="s">
+        <v>11</v>
+      </c>
+      <c r="E382" t="s">
+        <v>1703</v>
+      </c>
+      <c r="F382" t="s">
+        <v>1704</v>
+      </c>
+      <c r="G382" t="s">
+        <v>13</v>
+      </c>
+      <c r="H382" t="s">
+        <v>1704</v>
+      </c>
+      <c r="I382" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="383" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A383">
+        <v>382</v>
+      </c>
+      <c r="B383" t="s">
+        <v>1705</v>
+      </c>
+      <c r="C383" t="s">
+        <v>1706</v>
+      </c>
+      <c r="D383" t="s">
+        <v>11</v>
+      </c>
+      <c r="E383" t="s">
+        <v>1707</v>
+      </c>
+      <c r="F383" t="s">
+        <v>1708</v>
+      </c>
+      <c r="G383" t="s">
+        <v>487</v>
+      </c>
+      <c r="H383" t="s">
+        <v>1708</v>
+      </c>
+      <c r="I383" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="384" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A384">
+        <v>383</v>
+      </c>
+      <c r="B384" t="s">
+        <v>1709</v>
+      </c>
+      <c r="C384" t="s">
+        <v>917</v>
+      </c>
+      <c r="D384" t="s">
+        <v>32</v>
+      </c>
+      <c r="E384" t="s">
+        <v>1710</v>
+      </c>
+      <c r="F384" t="s">
+        <v>1711</v>
+      </c>
+      <c r="G384" t="s">
+        <v>13</v>
+      </c>
+      <c r="H384" t="s">
+        <v>1711</v>
+      </c>
+      <c r="I384" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="385" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A385">
+        <v>384</v>
+      </c>
+      <c r="B385" t="s">
+        <v>1712</v>
+      </c>
+      <c r="C385" t="s">
+        <v>1713</v>
+      </c>
+      <c r="D385" t="s">
+        <v>32</v>
+      </c>
+      <c r="E385" t="s">
+        <v>1714</v>
+      </c>
+      <c r="F385" t="s">
+        <v>1715</v>
+      </c>
+      <c r="G385" t="s">
+        <v>487</v>
+      </c>
+      <c r="H385" t="s">
+        <v>1715</v>
+      </c>
+      <c r="I385" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="386" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A386">
+        <v>385</v>
+      </c>
+      <c r="B386" t="s">
+        <v>1716</v>
+      </c>
+      <c r="C386" t="s">
+        <v>1717</v>
+      </c>
+      <c r="D386" t="s">
+        <v>32</v>
+      </c>
+      <c r="E386" t="s">
+        <v>1718</v>
+      </c>
+      <c r="F386" t="s">
+        <v>1719</v>
+      </c>
+      <c r="G386" t="s">
+        <v>487</v>
+      </c>
+      <c r="H386" t="s">
+        <v>1719</v>
+      </c>
+      <c r="I386" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="387" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A387">
+        <v>386</v>
+      </c>
+      <c r="B387" t="s">
+        <v>1720</v>
+      </c>
+      <c r="C387" t="s">
+        <v>1721</v>
+      </c>
+      <c r="D387" t="s">
+        <v>11</v>
+      </c>
+      <c r="E387" t="s">
+        <v>1722</v>
+      </c>
+      <c r="F387" t="s">
+        <v>1723</v>
+      </c>
+      <c r="G387" t="s">
+        <v>13</v>
+      </c>
+      <c r="H387" t="s">
+        <v>1723</v>
+      </c>
+      <c r="I387" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="388" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A388">
+        <v>387</v>
+      </c>
+      <c r="B388" t="s">
+        <v>1724</v>
+      </c>
+      <c r="C388" t="s">
+        <v>1725</v>
+      </c>
+      <c r="D388" t="s">
+        <v>32</v>
+      </c>
+      <c r="E388" t="s">
+        <v>1726</v>
+      </c>
+      <c r="F388" t="s">
+        <v>1727</v>
+      </c>
+      <c r="G388" t="s">
+        <v>487</v>
+      </c>
+      <c r="H388" t="s">
+        <v>1727</v>
+      </c>
+      <c r="I388" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="389" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A389">
+        <v>388</v>
+      </c>
+      <c r="B389" t="s">
+        <v>1728</v>
+      </c>
+      <c r="C389" t="s">
+        <v>1729</v>
+      </c>
+      <c r="D389" t="s">
+        <v>32</v>
+      </c>
+      <c r="E389" t="s">
+        <v>1730</v>
+      </c>
+      <c r="F389" t="s">
+        <v>1731</v>
+      </c>
+      <c r="G389" t="s">
+        <v>487</v>
+      </c>
+      <c r="H389" t="s">
+        <v>1731</v>
+      </c>
+      <c r="I389" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="390" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A390">
+        <v>389</v>
+      </c>
+      <c r="B390" t="s">
+        <v>1732</v>
+      </c>
+      <c r="C390" t="s">
+        <v>1733</v>
+      </c>
+      <c r="D390" t="s">
+        <v>32</v>
+      </c>
+      <c r="E390" t="s">
+        <v>1734</v>
+      </c>
+      <c r="F390" t="s">
+        <v>1735</v>
+      </c>
+      <c r="G390" t="s">
+        <v>13</v>
+      </c>
+      <c r="H390" t="s">
+        <v>1735</v>
+      </c>
+      <c r="I390" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="391" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A391">
+        <v>390</v>
+      </c>
+      <c r="B391" t="s">
+        <v>1736</v>
+      </c>
+      <c r="C391" t="s">
+        <v>1737</v>
+      </c>
+      <c r="D391" t="s">
+        <v>32</v>
+      </c>
+      <c r="E391" t="s">
+        <v>1738</v>
+      </c>
+      <c r="F391" t="s">
+        <v>1739</v>
+      </c>
+      <c r="G391" t="s">
+        <v>13</v>
+      </c>
+      <c r="H391" t="s">
+        <v>1739</v>
+      </c>
+      <c r="I391" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="392" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A392">
+        <v>391</v>
+      </c>
+      <c r="B392" t="s">
+        <v>1740</v>
+      </c>
+      <c r="C392" t="s">
+        <v>1741</v>
+      </c>
+      <c r="D392" t="s">
+        <v>32</v>
+      </c>
+      <c r="E392" t="s">
+        <v>1742</v>
+      </c>
+      <c r="F392" t="s">
+        <v>1743</v>
+      </c>
+      <c r="G392" t="s">
+        <v>487</v>
+      </c>
+      <c r="H392" t="s">
+        <v>1743</v>
+      </c>
+      <c r="I392" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="393" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A393">
+        <v>392</v>
+      </c>
+      <c r="B393" t="s">
+        <v>1744</v>
+      </c>
+      <c r="C393" t="s">
+        <v>1745</v>
+      </c>
+      <c r="D393" t="s">
+        <v>11</v>
+      </c>
+      <c r="E393" t="s">
+        <v>1746</v>
+      </c>
+      <c r="F393" t="s">
+        <v>1747</v>
+      </c>
+      <c r="G393" t="s">
+        <v>13</v>
+      </c>
+      <c r="H393" t="s">
+        <v>1747</v>
+      </c>
+      <c r="I393" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="394" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A394">
+        <v>393</v>
+      </c>
+      <c r="B394" t="s">
+        <v>1748</v>
+      </c>
+      <c r="C394" t="s">
+        <v>1749</v>
+      </c>
+      <c r="D394" t="s">
+        <v>32</v>
+      </c>
+      <c r="E394" t="s">
+        <v>1750</v>
+      </c>
+      <c r="F394" t="s">
+        <v>1751</v>
+      </c>
+      <c r="G394" t="s">
+        <v>13</v>
+      </c>
+      <c r="H394" t="s">
+        <v>1751</v>
+      </c>
+      <c r="I394" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="395" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A395">
+        <v>394</v>
+      </c>
+      <c r="B395" t="s">
+        <v>1752</v>
+      </c>
+      <c r="C395" t="s">
+        <v>1753</v>
+      </c>
+      <c r="D395" t="s">
+        <v>32</v>
+      </c>
+      <c r="E395" t="s">
+        <v>1754</v>
+      </c>
+      <c r="F395" t="s">
+        <v>1755</v>
+      </c>
+      <c r="G395" t="s">
+        <v>13</v>
+      </c>
+      <c r="H395" t="s">
+        <v>1755</v>
+      </c>
+      <c r="I395" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="396" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A396">
+        <v>395</v>
+      </c>
+      <c r="B396" t="s">
+        <v>1756</v>
+      </c>
+      <c r="C396" t="s">
+        <v>817</v>
+      </c>
+      <c r="D396" t="s">
+        <v>32</v>
+      </c>
+      <c r="E396" t="s">
+        <v>1757</v>
+      </c>
+      <c r="F396" t="s">
+        <v>1758</v>
+      </c>
+      <c r="G396" t="s">
+        <v>13</v>
+      </c>
+      <c r="H396" t="s">
+        <v>1758</v>
+      </c>
+      <c r="I396" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="397" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A397">
+        <v>396</v>
+      </c>
+      <c r="B397" t="s">
+        <v>1759</v>
+      </c>
+      <c r="C397" t="s">
+        <v>1760</v>
+      </c>
+      <c r="D397" t="s">
+        <v>32</v>
+      </c>
+      <c r="E397" t="s">
+        <v>1761</v>
+      </c>
+      <c r="F397" t="s">
+        <v>1762</v>
+      </c>
+      <c r="G397" t="s">
+        <v>13</v>
+      </c>
+      <c r="H397" t="s">
+        <v>1762</v>
+      </c>
+      <c r="I397" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="398" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A398">
+        <v>397</v>
+      </c>
+      <c r="B398" t="s">
+        <v>1763</v>
+      </c>
+      <c r="C398" t="s">
+        <v>1764</v>
+      </c>
+      <c r="D398" t="s">
+        <v>32</v>
+      </c>
+      <c r="E398" t="s">
+        <v>1765</v>
+      </c>
+      <c r="F398" t="s">
+        <v>1766</v>
+      </c>
+      <c r="G398" t="s">
+        <v>13</v>
+      </c>
+      <c r="H398" t="s">
+        <v>1766</v>
+      </c>
+      <c r="I398" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="399" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A399">
+        <v>398</v>
+      </c>
+      <c r="B399" t="s">
+        <v>1767</v>
+      </c>
+      <c r="C399" t="s">
+        <v>1768</v>
+      </c>
+      <c r="D399" t="s">
+        <v>32</v>
+      </c>
+      <c r="E399" t="s">
+        <v>1769</v>
+      </c>
+      <c r="F399" t="s">
+        <v>1770</v>
+      </c>
+      <c r="G399" t="s">
+        <v>13</v>
+      </c>
+      <c r="H399" t="s">
+        <v>1770</v>
+      </c>
+      <c r="I399" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="400" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A400">
+        <v>399</v>
+      </c>
+      <c r="B400" t="s">
+        <v>1771</v>
+      </c>
+      <c r="C400" t="s">
+        <v>1772</v>
+      </c>
+      <c r="D400" t="s">
+        <v>11</v>
+      </c>
+      <c r="E400" t="s">
+        <v>1773</v>
+      </c>
+      <c r="F400" t="s">
+        <v>1774</v>
+      </c>
+      <c r="G400" t="s">
+        <v>13</v>
+      </c>
+      <c r="H400" t="s">
+        <v>1774</v>
+      </c>
+      <c r="I400" t="s">
+        <v>1391</v>
+      </c>
+    </row>
+    <row r="401" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A401">
+        <v>400</v>
+      </c>
+      <c r="B401" t="s">
+        <v>1775</v>
+      </c>
+      <c r="C401" t="s">
+        <v>1776</v>
+      </c>
+      <c r="D401" t="s">
+        <v>11</v>
+      </c>
+      <c r="E401" t="s">
+        <v>1777</v>
+      </c>
+      <c r="F401" t="s">
+        <v>1778</v>
+      </c>
+      <c r="G401" t="s">
+        <v>13</v>
+      </c>
+      <c r="H401" t="s">
+        <v>1778</v>
+      </c>
+      <c r="I401" t="s">
+        <v>1391</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I301"/>
@@ -12727,7 +16803,7 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>1387</v>
+        <v>1779</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -12735,22 +16811,22 @@
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>1388</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>1389</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>1390</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>1391</v>
+        <v>1783</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -12758,12 +16834,12 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>1392</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>1393</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -12771,7 +16847,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>1394</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -12821,7 +16897,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>1395</v>
+        <v>1787</v>
       </c>
       <c r="B17" s="14">
         <f>SUM(B12:B14)</f>

</xml_diff>